<commit_message>
Sync embedded elevator tickets workbook
</commit_message>
<xml_diff>
--- a/textbook_examples/elevator_tickets.xlsx
+++ b/textbook_examples/elevator_tickets.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pjs998/Downloads/"/>
@@ -15,7 +15,23 @@
   <sheets>
     <sheet name="elevator_tickets" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -71,7 +87,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="18">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -928,9 +944,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D17671-FA6B-674F-BA45-D513988CF400}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -953,7 +969,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -976,7 +992,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
@@ -999,7 +1015,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1022,7 +1038,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1045,7 +1061,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1068,7 +1084,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1091,7 +1107,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1114,7 +1130,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1137,7 +1153,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1160,7 +1176,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1183,7 +1199,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1206,7 +1222,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1229,7 +1245,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1252,7 +1268,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1275,7 +1291,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1298,7 +1314,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1321,7 +1337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1344,7 +1360,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1367,7 +1383,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1390,7 +1406,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>20</v>
       </c>

</xml_diff>